<commit_message>
feat: push latest python data pipeline scripts
</commit_message>
<xml_diff>
--- a/Premium_Undervalued_Deals.xlsx
+++ b/Premium_Undervalued_Deals.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Deals of the Day" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="API Keys Blueprint" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -44,14 +44,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-        <bgColor rgb="001F4E78"/>
+        <fgColor rgb="007030A0"/>
+        <bgColor rgb="007030A0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
-        <bgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00F2F4F7"/>
+        <bgColor rgb="00F2F4F7"/>
       </patternFill>
     </fill>
   </fills>
@@ -73,15 +73,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -447,111 +444,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="57" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Property Address</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Current List Price</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Neighborhood Average</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Est. Discount %</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Market Status</t>
+          <t>Detected API Response Keys</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>123 Main St</t>
+          <t>ERROR: Vault credentials or data pull returned empty.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>$350,000</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>380000</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>7.9</v>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>789 Pine Rd</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>$420,000!!</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>450000</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>6.7</v>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>101 Maple Dr</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>$250,000</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>260000</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
+      <c r="B2" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>